<commit_message>
Labelling workbook: strict verdict/stage dropdowns, help pop-ups, note suggestions
openpyxl leaves the data-validation error alert off by default, so the
verdict and stage dropdowns accepted any typed value (E-013). Turn it on,
add input-message help per label column, a note-suggestion list (free
text allowed) and a "Dropdown options" sheet. Rebuilt with the same sample.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/evals/error_analysis/claims.xlsx
+++ b/evals/error_analysis/claims.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to label" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Claims" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dropdown options" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +37,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="3">
@@ -63,7 +68,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -80,6 +85,8 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -445,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -487,178 +494,190 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Step 1</t>
+          <t>Dropdowns</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Read the claim. What does it tell you?</t>
+          <t>Click a yellow cell: a short help pops up and an arrow opens the dropdown. human_verdict and human_stage accept only list values; human_note offers common reasons but you can type your own. Sheet 'Dropdown options' explains every value.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Step 2</t>
+          <t>Step 1</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Read the source and passage in 'evidence'. What is the source really about: which model, what size, pretraining or fine-tuning, text or speech?</t>
+          <t>Read the claim. What does it tell you?</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Step 3</t>
+          <t>Step 2</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Compare. Same thing, honestly stated: human_verdict = ok. Different thing, or overstated: wrong.</t>
+          <t>Read the source and passage in 'evidence'. What is the source really about: which model, what size, pretraining or fine-tuning, text or speech?</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Step 4 (only if wrong)</t>
+          <t>Step 3</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Find where it FIRST broke, walking source -&gt; fact -&gt; claim, and pick human_stage:</t>
+          <t>Compare. Same thing, honestly stated: human_verdict = ok. Different thing, or overstated: wrong.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>bad source</t>
+          <t>Step 4 (only if wrong)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>The source doesn't fit the goal (e.g. a speech model when the user said text only; a school essay-writing guide used as evidence about LLM reasoning).</t>
+          <t>Find where it FIRST broke, walking source -&gt; fact -&gt; claim, and pick human_stage:</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>extraction subject</t>
+          <t>bad source</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>The extracted fact (the 'FACT:' line) already names the wrong model, size or stage, or turns the source's statement into a general rule (often in the research question's words).</t>
+          <t>The source doesn't fit the goal (e.g. a speech model when the user said text only; a school essay-writing guide used as evidence about LLM reasoning).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>writing subject</t>
+          <t>extraction subject</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>The fact is right, but the report sentence drops or changes what it is about (e.g. one project's settings presented as what 'the model' must do).</t>
+          <t>The extracted fact (the 'FACT:' line) already names the wrong model, size or stage, or turns the source's statement into a general rule (often in the research question's words).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>writing stitch</t>
+          <t>writing subject</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Facts from different sources merged into one claim that none of them makes.</t>
+          <t>The fact is right, but the report sentence drops or changes what it is about (e.g. one project's settings presented as what 'the model' must do).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>writing stitch</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Content fine, evidence label wrong: 'established' needs two or more documents saying the same thing; a recommendation drawn from one source is an inference, not 'single source'.</t>
+          <t>Facts from different sources merged into one claim that none of them makes.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>retrieval miss / other</t>
+          <t>label</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Retrieval miss = the right source was never found (rare for a cited claim). Other = anything else; say what in human_note.</t>
+          <t>Content fine, evidence label wrong: 'established' needs two or more documents saying the same thing; a recommendation drawn from one source is an inference, not 'single source'.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Worked example: C34</t>
+          <t>retrieval miss / other</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Claim: 'use optimal hyperparameters for a 4B model: batch size 4 [E7], weight decay 0.001 [E8]', labelled established. Source: an appendix table in a paper about EVALUATING POST-TRAINED models; nothing about pretraining a 4B model. Fact E7: 'optimal hyperparameters for pretraining a 4B model include batch size 4': already wrong. Verdict: wrong. Stage: extraction subject (the first break is the fact; the claim only repeats it).</t>
+          <t>Retrieval miss = the right source was never found (rare for a cited claim). Other = anything else; say what in human_note.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Tip: 'the model'</t>
+          <t>Worked example: C34</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>If a claim says 'the model' or 'this process', check the sentence before it in the report (claims.md, or the report itself): often the subject was named there, and then the claim is ok.</t>
+          <t>Claim: 'use optimal hyperparameters for a 4B model: batch size 4 [E7], weight decay 0.001 [E8]', labelled established. Source: an appendix table in a paper about EVALUATING POST-TRAINED models; nothing about pretraining a 4B model. Fact E7: 'optimal hyperparameters for pretraining a 4B model include batch size 4': already wrong. Verdict: wrong. Stage: extraction subject (the first break is the fact; the claim only repeats it).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Tip: weak relevance</t>
+          <t>Tip: 'the model'</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>True but only weakly relevant (e.g. it names a 295B frontier model in a 4B-8B report): ok, with a note. Use wrong only when the sentence would actually mislead.</t>
+          <t>If a claim says 'the model' or 'this process', check the sentence before it in the report (claims.md, or the report itself): often the subject was named there, and then the claim is ok.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Blind labelling</t>
+          <t>Tip: weak relevance</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Don't open claude_labels.csv (or its commit) until you are done; the agreement score depends on it.</t>
+          <t>True but only weakly relevant (e.g. it names a 295B frontier model in a 4B-8B report): ok, with a note. Use wrong only when the sentence would actually mislead.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
+          <t>Blind labelling</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Don't open claude_labels.csv (or its commit) until you are done; the agreement score depends on it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
           <t>When done</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Save the workbook (keep .xlsx), then run: python scripts/error_analysis.py tally</t>
         </is>
@@ -2713,14 +2732,347 @@
       <c r="I51" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="G2:G51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a valid label" error="Pick a value from the list" type="list">
-      <formula1>"ok,wrong"</formula1>
+  <dataValidations count="3">
+    <dataValidation sqref="G2:G51" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid label" error="Pick a value from the list (meanings on 'Dropdown options')" promptTitle="Verdict (required)" prompt="ok = the sentence honestly says what its source says. wrong = it would mislead you (wrong model/size/stage, off-goal, overstated, mislabelled)." type="list">
+      <formula1>'Dropdown options'!$A$2:$A$3</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not a valid label" error="Pick a value from the list" type="list">
-      <formula1>"retrieval miss,bad source,extraction subject,writing subject,writing stitch,label,other"</formula1>
+    <dataValidation sqref="H2:H51" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not a valid label" error="Pick a value from the list (meanings on 'Dropdown options')" promptTitle="Stage (only if wrong)" prompt="First check that fails: 1 bad source, 2 extraction subject (FACT wrong), 3 writing subject (claim changes the fact), 4 writing stitch, 5 label. Else retrieval miss / other. Empty if ok." type="list">
+      <formula1>'Dropdown options'!$A$6:$A$12</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I51" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Note (optional)" prompt="Pick a common reason or type your own words. Useful for wrong, borderline or weakly relevant rows." type="list">
+      <formula1>'Dropdown options'!$A$15:$A$28</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>human_verdict</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>The sentence honestly says what its source says, about the right thing</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>wrong</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>The sentence would mislead a reader: wrong model, size or stage, off-goal source, overstated, or mislabelled</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>human_stage</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>bad source</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>1st check: the source does not fit the goal (speech model for a text goal, essay guide)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>extraction subject</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2nd check: the FACT line already names the wrong model, size or stage, or turns the source into a general rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>writing subject</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>3rd check: the fact is right, the claim drops or changes its subject or meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>writing stitch</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>4th check: facts from different sources merged into a claim none of them makes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>5th check: content fine, evidence label wrong ('established' needs 2+ documents)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>retrieval miss</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>The right source was never found (rare for a cited claim)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>None of the above; say what in human_note</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>human_note</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>wrong model</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>The fact or claim names a different model than the source</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>wrong size</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Parameter count does not match the source</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>fine-tuning presented as pretraining</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>A fine-tune's settings or hardware read as pretraining</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>post-training presented as pretraining</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>A post-training study's numbers read as pretraining</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>speech source, goal is text</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>ASR / speech translation used for a text-only goal</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>off-goal source</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>The document is not about the goal at all</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>one project's settings as a general rule</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>What one project did, stated as what you must do</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>benchmark rule as a model requirement</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>A test-harness rule stated as a property of the model</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>overstated</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>The source says less, or says it more cautiously</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>merges different sources</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Two sources combined into something neither says</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>'established' on one document</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Label needs two or more documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>true but weak relevance</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Correct, but far from the goal (e.g. a 295B model in a 4B-8B report)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>subject named in the sentence before</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>'The model' is fine once you read the previous sentence</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Could go either way</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>